<commit_message>
Corrección del Código Postal y su seguridad.
</commit_message>
<xml_diff>
--- a/ANDESMAR.xlsx
+++ b/ANDESMAR.xlsx
@@ -42,9 +42,6 @@
     <t>TELEFONO:</t>
   </si>
   <si>
-    <t>DETALLE:</t>
-  </si>
-  <si>
     <t>CIUDAD / PUEBLO:</t>
   </si>
   <si>
@@ -58,6 +55,9 @@
   </si>
   <si>
     <t>FULANO</t>
+  </si>
+  <si>
+    <t>CODIGO POSTAL:</t>
   </si>
 </sst>
 </file>
@@ -972,7 +972,7 @@
       <c r="C7" s="21"/>
       <c r="D7" s="8"/>
       <c r="E7" s="46" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F7" s="47"/>
       <c r="G7" s="47"/>
@@ -989,7 +989,7 @@
       <c r="C8" s="21"/>
       <c r="D8" s="10"/>
       <c r="E8" s="28" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F8" s="29"/>
       <c r="G8" s="29"/>
@@ -1035,12 +1035,12 @@
     <row r="11" spans="1:11" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="9"/>
       <c r="B11" s="40" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C11" s="41"/>
       <c r="D11" s="12"/>
       <c r="E11" s="31" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F11" s="32"/>
       <c r="G11" s="32"/>
@@ -1057,7 +1057,7 @@
       <c r="C12" s="43"/>
       <c r="D12" s="10"/>
       <c r="E12" s="34" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F12" s="35"/>
       <c r="G12" s="35"/>
@@ -1069,11 +1069,13 @@
     <row r="13" spans="1:11" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="9"/>
       <c r="B13" s="44" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C13" s="45"/>
       <c r="D13" s="12"/>
-      <c r="E13" s="37"/>
+      <c r="E13" s="37">
+        <v>5001</v>
+      </c>
       <c r="F13" s="38"/>
       <c r="G13" s="38"/>
       <c r="H13" s="38"/>
@@ -1100,7 +1102,7 @@
       <c r="C15" s="14"/>
       <c r="D15" s="14"/>
       <c r="E15" s="25" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F15" s="25"/>
       <c r="G15" s="25"/>
@@ -1137,6 +1139,7 @@
     </row>
     <row r="18" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="16">
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="B1:J5"/>

</xml_diff>